<commit_message>
2.1.12: Ignore NotNull if ignoreAnnotation is specivied.
</commit_message>
<xml_diff>
--- a/meta/objects/BlancoValueObjectAnnotationSample.xlsx
+++ b/meta/objects/BlancoValueObjectAnnotationSample.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10812"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10911"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tueda/data/webstorm/blanco/blancoValueObject/meta/objects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC996B5-AFE3-1141-B4F2-8DB588757E02}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9023E36E-85DD-8541-B100-A894727B7A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="660" yWindow="500" windowWidth="25520" windowHeight="15540" tabRatio="640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,6 @@
     <sheet name="valueObject" sheetId="1" r:id="rId1"/>
     <sheet name="config" sheetId="2" r:id="rId2"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
   <definedNames>
     <definedName name="accessScope">config!$B$4:$B$6</definedName>
     <definedName name="accessScope2">config!$B$4:$B$5</definedName>
@@ -44,7 +41,7 @@
     <definedName name="必須" localSheetId="1">#REF!</definedName>
     <definedName name="必須">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
@@ -62,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="57">
   <si>
     <t>クラス名</t>
   </si>
@@ -316,6 +313,17 @@
   <si>
     <t>フィールド名の変形</t>
     <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>必須</t>
+    <rPh sb="0" eb="2">
+      <t xml:space="preserve">ヒッス </t>
+    </rPh>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>○</t>
+    <phoneticPr fontId="4"/>
   </si>
 </sst>
 </file>
@@ -999,27 +1007,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1048,6 +1035,27 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1134,21 +1142,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="valueObject"/>
-      <sheetName val="config"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1476,37 +1469,37 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
-    <col min="2" max="6" width="23.5" style="1" customWidth="1"/>
-    <col min="7" max="7" width="13.1640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="6.83203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="28" style="1" customWidth="1"/>
-    <col min="10" max="10" width="33.33203125" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="9" style="1"/>
+    <col min="2" max="7" width="23.5" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="6.83203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="28" style="1" customWidth="1"/>
+    <col min="11" max="11" width="33.33203125" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="19">
+    <row r="1" spans="1:12" ht="19">
       <c r="A1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:12">
       <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:12">
       <c r="B3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:12">
       <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
@@ -1515,8 +1508,9 @@
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="5"/>
-    </row>
-    <row r="6" spans="1:11">
+      <c r="G5" s="5"/>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" s="3" t="s">
         <v>0</v>
       </c>
@@ -1527,9 +1521,10 @@
       <c r="D6" s="12"/>
       <c r="E6" s="12"/>
       <c r="F6" s="8"/>
-      <c r="G6" s="9"/>
-    </row>
-    <row r="7" spans="1:11">
+      <c r="G6" s="8"/>
+      <c r="H6" s="9"/>
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" s="3" t="s">
         <v>1</v>
       </c>
@@ -1540,9 +1535,10 @@
       <c r="D7" s="37"/>
       <c r="E7" s="37"/>
       <c r="F7" s="11"/>
-      <c r="G7" s="9"/>
-    </row>
-    <row r="8" spans="1:11">
+      <c r="G7" s="11"/>
+      <c r="H7" s="9"/>
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8" s="3" t="s">
         <v>23</v>
       </c>
@@ -1553,9 +1549,10 @@
       <c r="D8" s="37"/>
       <c r="E8" s="37"/>
       <c r="F8" s="11"/>
-      <c r="G8" s="9"/>
-    </row>
-    <row r="9" spans="1:11">
+      <c r="G8" s="11"/>
+      <c r="H8" s="9"/>
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9" s="3" t="s">
         <v>27</v>
       </c>
@@ -1566,24 +1563,26 @@
       <c r="D9" s="37"/>
       <c r="E9" s="37"/>
       <c r="F9" s="11"/>
-      <c r="G9" s="41"/>
-    </row>
-    <row r="10" spans="1:11" ht="29" customHeight="1">
+      <c r="G9" s="11"/>
+      <c r="H9" s="41"/>
+    </row>
+    <row r="10" spans="1:12" ht="29" customHeight="1">
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B10" s="6"/>
-      <c r="C10" s="60" t="s">
+      <c r="C10" s="72" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="61"/>
-      <c r="E10" s="61"/>
-      <c r="F10" s="62"/>
-      <c r="G10" s="38"/>
+      <c r="D10" s="73"/>
+      <c r="E10" s="73"/>
+      <c r="F10" s="73"/>
+      <c r="G10" s="74"/>
       <c r="H10" s="38"/>
       <c r="I10" s="38"/>
-    </row>
-    <row r="11" spans="1:11">
+      <c r="J10" s="38"/>
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11" s="3" t="s">
         <v>3</v>
       </c>
@@ -1594,37 +1593,40 @@
       <c r="D11" s="12"/>
       <c r="E11" s="12"/>
       <c r="F11" s="8"/>
-      <c r="G11" s="38"/>
+      <c r="G11" s="8"/>
       <c r="H11" s="38"/>
       <c r="I11" s="38"/>
-    </row>
-    <row r="12" spans="1:11" s="33" customFormat="1">
-      <c r="A12" s="76" t="s">
+      <c r="J11" s="38"/>
+    </row>
+    <row r="12" spans="1:12" s="33" customFormat="1">
+      <c r="A12" s="69" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="77"/>
-      <c r="C12" s="78" t="s">
+      <c r="B12" s="70"/>
+      <c r="C12" s="71" t="s">
         <v>53</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
       <c r="F12"/>
       <c r="G12"/>
-    </row>
-    <row r="13" spans="1:11" s="33" customFormat="1">
-      <c r="A13" s="76" t="s">
+      <c r="H12"/>
+    </row>
+    <row r="13" spans="1:12" s="33" customFormat="1">
+      <c r="A13" s="69" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="77"/>
-      <c r="C13" s="78" t="s">
+      <c r="B13" s="70"/>
+      <c r="C13" s="71" t="s">
         <v>53</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
       <c r="F13"/>
       <c r="G13"/>
-    </row>
-    <row r="14" spans="1:11" s="43" customFormat="1">
+      <c r="H13"/>
+    </row>
+    <row r="14" spans="1:12" s="43" customFormat="1">
       <c r="A14" s="38"/>
       <c r="B14" s="42"/>
       <c r="C14" s="38"/>
@@ -1634,8 +1636,9 @@
       <c r="G14" s="38"/>
       <c r="H14" s="38"/>
       <c r="I14" s="38"/>
-    </row>
-    <row r="15" spans="1:11">
+      <c r="J14" s="38"/>
+    </row>
+    <row r="15" spans="1:12">
       <c r="A15" s="31" t="s">
         <v>18</v>
       </c>
@@ -1644,13 +1647,14 @@
       <c r="D15" s="32"/>
       <c r="E15" s="32"/>
       <c r="F15" s="32"/>
-      <c r="G15" s="39"/>
-      <c r="H15" s="33"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="39"/>
       <c r="I15" s="33"/>
       <c r="J15" s="33"/>
       <c r="K15" s="33"/>
-    </row>
-    <row r="16" spans="1:11">
+      <c r="L15" s="33"/>
+    </row>
+    <row r="16" spans="1:12">
       <c r="A16" s="34" t="s">
         <v>0</v>
       </c>
@@ -1659,13 +1663,14 @@
       <c r="D16" s="36"/>
       <c r="E16" s="36"/>
       <c r="F16" s="36"/>
-      <c r="G16" s="40"/>
-      <c r="H16" s="33"/>
+      <c r="G16" s="36"/>
+      <c r="H16" s="40"/>
       <c r="I16" s="33"/>
       <c r="J16" s="33"/>
       <c r="K16" s="33"/>
-    </row>
-    <row r="17" spans="1:11">
+      <c r="L16" s="33"/>
+    </row>
+    <row r="17" spans="1:12">
       <c r="A17" s="3" t="s">
         <v>25</v>
       </c>
@@ -1674,9 +1679,10 @@
       <c r="D17" s="37"/>
       <c r="E17" s="37"/>
       <c r="F17" s="11"/>
-      <c r="G17" s="9"/>
-    </row>
-    <row r="18" spans="1:11">
+      <c r="G17" s="11"/>
+      <c r="H17" s="9"/>
+    </row>
+    <row r="18" spans="1:12">
       <c r="A18" s="3" t="s">
         <v>23</v>
       </c>
@@ -1685,9 +1691,10 @@
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
       <c r="F18" s="8"/>
-      <c r="G18" s="9"/>
-    </row>
-    <row r="19" spans="1:11">
+      <c r="G18" s="8"/>
+      <c r="H18" s="9"/>
+    </row>
+    <row r="19" spans="1:12">
       <c r="A19" s="13"/>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
@@ -1696,8 +1703,9 @@
       <c r="F19" s="13"/>
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
-    </row>
-    <row r="20" spans="1:11">
+      <c r="I19" s="13"/>
+    </row>
+    <row r="20" spans="1:12">
       <c r="A20" s="31" t="s">
         <v>38</v>
       </c>
@@ -1706,13 +1714,14 @@
       <c r="D20" s="32"/>
       <c r="E20" s="32"/>
       <c r="F20" s="32"/>
-      <c r="G20" s="39"/>
-      <c r="H20" s="49"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="39"/>
       <c r="I20" s="49"/>
       <c r="J20" s="49"/>
       <c r="K20" s="49"/>
-    </row>
-    <row r="21" spans="1:11">
+      <c r="L20" s="49"/>
+    </row>
+    <row r="21" spans="1:12">
       <c r="A21" s="54" t="s">
         <v>39</v>
       </c>
@@ -1723,13 +1732,14 @@
       <c r="D21" s="48"/>
       <c r="E21" s="48"/>
       <c r="F21" s="35"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="50"/>
-      <c r="I21" s="51"/>
+      <c r="G21" s="35"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="50"/>
       <c r="J21" s="51"/>
-      <c r="K21" s="41"/>
-    </row>
-    <row r="22" spans="1:11">
+      <c r="K21" s="51"/>
+      <c r="L21" s="41"/>
+    </row>
+    <row r="22" spans="1:12">
       <c r="A22" s="58">
         <v>1</v>
       </c>
@@ -1740,39 +1750,42 @@
       <c r="D22" s="44"/>
       <c r="E22" s="44"/>
       <c r="F22" s="45"/>
-      <c r="G22" s="52"/>
-      <c r="H22" s="42"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="52"/>
       <c r="I22" s="42"/>
       <c r="J22" s="42"/>
-      <c r="K22" s="41"/>
-    </row>
-    <row r="23" spans="1:11">
+      <c r="K22" s="42"/>
+      <c r="L22" s="41"/>
+    </row>
+    <row r="23" spans="1:12">
       <c r="A23" s="58"/>
       <c r="B23" s="53"/>
       <c r="C23" s="46"/>
       <c r="D23" s="46"/>
       <c r="E23" s="46"/>
       <c r="F23" s="47"/>
-      <c r="G23" s="52"/>
-      <c r="H23" s="42"/>
+      <c r="G23" s="47"/>
+      <c r="H23" s="52"/>
       <c r="I23" s="42"/>
       <c r="J23" s="42"/>
-      <c r="K23" s="41"/>
-    </row>
-    <row r="24" spans="1:11">
+      <c r="K23" s="42"/>
+      <c r="L23" s="41"/>
+    </row>
+    <row r="24" spans="1:12">
       <c r="A24" s="59"/>
       <c r="B24" s="55"/>
       <c r="C24" s="56"/>
       <c r="D24" s="56"/>
       <c r="E24" s="56"/>
       <c r="F24" s="57"/>
-      <c r="G24" s="52"/>
-      <c r="H24" s="42"/>
+      <c r="G24" s="57"/>
+      <c r="H24" s="52"/>
       <c r="I24" s="42"/>
       <c r="J24" s="42"/>
-      <c r="K24" s="41"/>
-    </row>
-    <row r="25" spans="1:11">
+      <c r="K24" s="42"/>
+      <c r="L24" s="41"/>
+    </row>
+    <row r="25" spans="1:12">
       <c r="A25" s="13"/>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
@@ -1781,8 +1794,9 @@
       <c r="F25" s="13"/>
       <c r="G25" s="13"/>
       <c r="H25" s="13"/>
-    </row>
-    <row r="26" spans="1:11">
+      <c r="I25" s="13"/>
+    </row>
+    <row r="26" spans="1:12">
       <c r="A26" s="3" t="s">
         <v>11</v>
       </c>
@@ -1794,50 +1808,55 @@
       <c r="G26" s="14"/>
       <c r="H26" s="14"/>
       <c r="I26" s="14"/>
-      <c r="J26" s="6"/>
-      <c r="K26" s="15"/>
-    </row>
-    <row r="27" spans="1:11" ht="13.5" customHeight="1">
-      <c r="A27" s="64" t="s">
+      <c r="J26" s="14"/>
+      <c r="K26" s="6"/>
+      <c r="L26" s="15"/>
+    </row>
+    <row r="27" spans="1:12" ht="13.5" customHeight="1">
+      <c r="A27" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="64" t="s">
+      <c r="B27" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="C27" s="63" t="s">
+      <c r="C27" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="D27" s="63" t="s">
+      <c r="D27" s="75" t="s">
         <v>21</v>
       </c>
-      <c r="E27" s="65" t="s">
+      <c r="E27" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="F27" s="63" t="s">
+      <c r="F27" s="75" t="s">
         <v>6</v>
       </c>
-      <c r="G27" s="63" t="s">
+      <c r="G27" s="75" t="s">
+        <v>55</v>
+      </c>
+      <c r="H27" s="75" t="s">
         <v>2</v>
       </c>
-      <c r="H27" s="63"/>
-      <c r="I27" s="16"/>
-      <c r="J27" s="17"/>
-      <c r="K27" s="9"/>
-    </row>
-    <row r="28" spans="1:11">
-      <c r="A28" s="64"/>
-      <c r="B28" s="64"/>
-      <c r="C28" s="63"/>
-      <c r="D28" s="63"/>
-      <c r="E28" s="66"/>
-      <c r="F28" s="63"/>
-      <c r="G28" s="63"/>
-      <c r="H28" s="63"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="30"/>
-      <c r="K28" s="15"/>
-    </row>
-    <row r="29" spans="1:11">
+      <c r="I27" s="75"/>
+      <c r="J27" s="16"/>
+      <c r="K27" s="17"/>
+      <c r="L27" s="9"/>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" s="76"/>
+      <c r="B28" s="76"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="75"/>
+      <c r="E28" s="78"/>
+      <c r="F28" s="75"/>
+      <c r="G28" s="75"/>
+      <c r="H28" s="75"/>
+      <c r="I28" s="75"/>
+      <c r="J28" s="18"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="15"/>
+    </row>
+    <row r="29" spans="1:12">
       <c r="A29" s="19">
         <v>1</v>
       </c>
@@ -1853,14 +1872,17 @@
         <v>42</v>
       </c>
       <c r="G29" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="H29" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="H29" s="22"/>
       <c r="I29" s="22"/>
-      <c r="J29" s="29"/>
-      <c r="K29" s="15"/>
-    </row>
-    <row r="30" spans="1:11">
+      <c r="J29" s="22"/>
+      <c r="K29" s="29"/>
+      <c r="L29" s="15"/>
+    </row>
+    <row r="30" spans="1:12">
       <c r="A30" s="19">
         <v>2</v>
       </c>
@@ -1875,15 +1897,16 @@
       </c>
       <c r="E30" s="21"/>
       <c r="F30" s="21"/>
-      <c r="G30" s="21" t="s">
+      <c r="G30" s="21"/>
+      <c r="H30" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="H30" s="22"/>
       <c r="I30" s="22"/>
-      <c r="J30" s="23"/>
-      <c r="K30" s="15"/>
-    </row>
-    <row r="31" spans="1:11">
+      <c r="J30" s="22"/>
+      <c r="K30" s="23"/>
+      <c r="L30" s="15"/>
+    </row>
+    <row r="31" spans="1:12">
       <c r="A31" s="19">
         <v>3</v>
       </c>
@@ -1898,15 +1921,16 @@
         <v>34</v>
       </c>
       <c r="F31" s="21"/>
-      <c r="G31" s="21" t="s">
+      <c r="G31" s="21"/>
+      <c r="H31" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="H31" s="22"/>
       <c r="I31" s="22"/>
-      <c r="J31" s="23"/>
-      <c r="K31" s="15"/>
-    </row>
-    <row r="32" spans="1:11">
+      <c r="J31" s="22"/>
+      <c r="K31" s="23"/>
+      <c r="L31" s="15"/>
+    </row>
+    <row r="32" spans="1:12">
       <c r="A32" s="19">
         <v>4</v>
       </c>
@@ -1921,15 +1945,16 @@
         <v>32</v>
       </c>
       <c r="F32" s="21"/>
-      <c r="G32" s="21" t="s">
+      <c r="G32" s="21"/>
+      <c r="H32" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="H32" s="22"/>
       <c r="I32" s="22"/>
-      <c r="J32" s="23"/>
-      <c r="K32" s="15"/>
-    </row>
-    <row r="33" spans="1:11">
+      <c r="J32" s="22"/>
+      <c r="K32" s="23"/>
+      <c r="L32" s="15"/>
+    </row>
+    <row r="33" spans="1:12">
       <c r="A33" s="24"/>
       <c r="B33" s="25"/>
       <c r="C33" s="26"/>
@@ -1937,25 +1962,27 @@
       <c r="E33" s="26"/>
       <c r="F33" s="26"/>
       <c r="G33" s="26"/>
-      <c r="H33" s="27"/>
+      <c r="H33" s="26"/>
       <c r="I33" s="27"/>
-      <c r="J33" s="28"/>
-      <c r="K33" s="15"/>
+      <c r="J33" s="27"/>
+      <c r="K33" s="28"/>
+      <c r="L33" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="G27:H28"/>
+  <mergeCells count="9">
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="H27:I28"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="B27:B28"/>
     <mergeCell ref="C27:C28"/>
-    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="G27:G28"/>
     <mergeCell ref="D27:D28"/>
     <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
   </mergeCells>
   <phoneticPr fontId="4"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F49" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F49:G49" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>型</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1982,78 +2009,78 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="3" width="8.83203125" style="69" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" style="69" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" style="69" customWidth="1"/>
-    <col min="6" max="6" width="18.5" style="69" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.83203125" style="69" customWidth="1"/>
-    <col min="8" max="8" width="18.6640625" style="69" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.83203125" style="69" customWidth="1"/>
-    <col min="10" max="10" width="18.6640625" style="69" bestFit="1" customWidth="1"/>
-    <col min="11" max="256" width="8.83203125" style="69" customWidth="1"/>
-    <col min="257" max="16384" width="10.83203125" style="69"/>
+    <col min="1" max="3" width="8.83203125" style="62" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" style="62" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" style="62" customWidth="1"/>
+    <col min="6" max="6" width="18.5" style="62" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.83203125" style="62" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" style="62" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.83203125" style="62" customWidth="1"/>
+    <col min="10" max="10" width="18.6640625" style="62" bestFit="1" customWidth="1"/>
+    <col min="11" max="256" width="8.83203125" style="62" customWidth="1"/>
+    <col min="257" max="16384" width="10.83203125" style="62"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="19">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="60" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="68" t="s">
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="61" t="s">
         <v>44</v>
       </c>
-      <c r="M1" s="68"/>
+      <c r="M1" s="61"/>
     </row>
     <row r="3" spans="1:13">
-      <c r="B3" s="70" t="s">
+      <c r="B3" s="63" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="70" t="s">
+      <c r="D3" s="63" t="s">
         <v>46</v>
       </c>
-      <c r="F3" s="70" t="s">
+      <c r="F3" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="H3" s="70" t="s">
+      <c r="H3" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="J3" s="70" t="s">
+      <c r="J3" s="63" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="B4" s="71"/>
-      <c r="D4" s="72"/>
-      <c r="F4" s="72"/>
-      <c r="H4" s="72"/>
-      <c r="J4" s="72"/>
+      <c r="B4" s="64"/>
+      <c r="D4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="J4" s="65"/>
     </row>
     <row r="5" spans="1:13">
-      <c r="B5" s="73" t="s">
+      <c r="B5" s="66" t="s">
         <v>50</v>
       </c>
-      <c r="D5" s="74" t="s">
+      <c r="D5" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="F5" s="74" t="s">
+      <c r="F5" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="H5" s="74" t="s">
+      <c r="H5" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="J5" s="74" t="s">
+      <c r="J5" s="67" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="B6" s="75"/>
+      <c r="B6" s="68"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4"/>

</xml_diff>